<commit_message>
Auto update data 2026/03/19 週四
</commit_message>
<xml_diff>
--- a/rebalance_holdings_final.xlsx
+++ b/rebalance_holdings_final.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I236"/>
+  <dimension ref="A1:I237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11518,6 +11518,53 @@
       <c r="I236" t="inlineStr">
         <is>
           <t>22.46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>27.27%</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>24.93%</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>24.57%</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>20.08%</t>
         </is>
       </c>
     </row>
@@ -11532,7 +11579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO236"/>
+  <dimension ref="A1:AO237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50985,6 +51032,173 @@
       </c>
       <c r="AO236" t="n">
         <v>0.5001</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>1.4668</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>1.0385</v>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="G237" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="I237" t="n">
+        <v>0.9524</v>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="K237" t="n">
+        <v>0.702</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>FCX</t>
+        </is>
+      </c>
+      <c r="M237" t="n">
+        <v>0.642</v>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="O237" t="n">
+        <v>0.629</v>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>TPL</t>
+        </is>
+      </c>
+      <c r="Q237" t="n">
+        <v>0.6185</v>
+      </c>
+      <c r="R237" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="S237" t="n">
+        <v>0.6171</v>
+      </c>
+      <c r="T237" t="inlineStr">
+        <is>
+          <t>LMT</t>
+        </is>
+      </c>
+      <c r="U237" t="n">
+        <v>0.5862000000000001</v>
+      </c>
+      <c r="V237" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="W237" t="n">
+        <v>0.5685</v>
+      </c>
+      <c r="X237" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="Y237" t="n">
+        <v>0.5652</v>
+      </c>
+      <c r="Z237" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="AA237" t="n">
+        <v>0.5423</v>
+      </c>
+      <c r="AB237" t="inlineStr">
+        <is>
+          <t>ALB</t>
+        </is>
+      </c>
+      <c r="AC237" t="n">
+        <v>0.5204</v>
+      </c>
+      <c r="AD237" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="AE237" t="n">
+        <v>0.5196</v>
+      </c>
+      <c r="AF237" t="inlineStr">
+        <is>
+          <t>KEYS</t>
+        </is>
+      </c>
+      <c r="AG237" t="n">
+        <v>0.5149</v>
+      </c>
+      <c r="AH237" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+      <c r="AI237" t="n">
+        <v>0.5111</v>
+      </c>
+      <c r="AJ237" t="inlineStr">
+        <is>
+          <t>ODFL</t>
+        </is>
+      </c>
+      <c r="AK237" t="n">
+        <v>0.5032</v>
+      </c>
+      <c r="AL237" t="inlineStr">
+        <is>
+          <t>FDX</t>
+        </is>
+      </c>
+      <c r="AM237" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="AN237" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
+      <c r="AO237" t="n">
+        <v>0.4727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update data 2026/03/20 週五
</commit_message>
<xml_diff>
--- a/rebalance_holdings_final.xlsx
+++ b/rebalance_holdings_final.xlsx
@@ -41174,11 +41174,11 @@
       </c>
       <c r="AN177" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>HWM</t>
         </is>
       </c>
       <c r="AO177" t="n">
-        <v>0.3248</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="178">
@@ -41309,43 +41309,43 @@
       </c>
       <c r="AF178" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="AG178" t="n">
-        <v>0.3382</v>
+        <v>0.3279</v>
       </c>
       <c r="AH178" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="AI178" t="n">
-        <v>0.3279</v>
+        <v>0.3111</v>
       </c>
       <c r="AJ178" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>DAY</t>
         </is>
       </c>
       <c r="AK178" t="n">
-        <v>0.3111</v>
+        <v>0.3087</v>
       </c>
       <c r="AL178" t="inlineStr">
         <is>
-          <t>DAY</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="AM178" t="n">
-        <v>0.3087</v>
+        <v>0.3057</v>
       </c>
       <c r="AN178" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>TRGP</t>
         </is>
       </c>
       <c r="AO178" t="n">
-        <v>0.3057</v>
+        <v>0.3024</v>
       </c>
     </row>
     <row r="179">
@@ -41460,59 +41460,59 @@
       </c>
       <c r="AB179" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="AC179" t="n">
-        <v>0.3448</v>
+        <v>0.3432</v>
       </c>
       <c r="AD179" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="AE179" t="n">
-        <v>0.3432</v>
+        <v>0.3392</v>
       </c>
       <c r="AF179" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>FFIV</t>
         </is>
       </c>
       <c r="AG179" t="n">
-        <v>0.3392</v>
+        <v>0.3312</v>
       </c>
       <c r="AH179" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>CBRE</t>
         </is>
       </c>
       <c r="AI179" t="n">
-        <v>0.3312</v>
+        <v>0.3282</v>
       </c>
       <c r="AJ179" t="inlineStr">
         <is>
-          <t>CBRE</t>
+          <t>NCLH</t>
         </is>
       </c>
       <c r="AK179" t="n">
-        <v>0.3282</v>
+        <v>0.3177</v>
       </c>
       <c r="AL179" t="inlineStr">
         <is>
-          <t>NCLH</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="AM179" t="n">
-        <v>0.3177</v>
+        <v>0.3151</v>
       </c>
       <c r="AN179" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>GILD</t>
         </is>
       </c>
       <c r="AO179" t="n">
-        <v>0.3151</v>
+        <v>0.3146</v>
       </c>
     </row>
     <row r="180">
@@ -43838,19 +43838,19 @@
       </c>
       <c r="AL193" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>META</t>
         </is>
       </c>
       <c r="AM193" t="n">
-        <v>0.1996</v>
+        <v>0.1887</v>
       </c>
       <c r="AN193" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>WMT</t>
         </is>
       </c>
       <c r="AO193" t="n">
-        <v>0.1887</v>
+        <v>0.1701</v>
       </c>
     </row>
     <row r="194">

</xml_diff>

<commit_message>
Auto update data 2026/04/16 週四
</commit_message>
<xml_diff>
--- a/rebalance_holdings_final.xlsx
+++ b/rebalance_holdings_final.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I237"/>
+  <dimension ref="A1:I238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11565,6 +11565,53 @@
       <c r="I237" t="inlineStr">
         <is>
           <t>20.08%</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>28.91%</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>24.61%</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>24.44%</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>22.03%</t>
         </is>
       </c>
     </row>
@@ -11579,7 +11626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO237"/>
+  <dimension ref="A1:AO238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51199,6 +51246,173 @@
       </c>
       <c r="AO237" t="n">
         <v>0.4727</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>0.8643</v>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="G238" t="n">
+        <v>0.8406</v>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="I238" t="n">
+        <v>0.8351</v>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="K238" t="n">
+        <v>0.8096</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="M238" t="n">
+        <v>0.7869</v>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="O238" t="n">
+        <v>0.7521</v>
+      </c>
+      <c r="P238" t="inlineStr">
+        <is>
+          <t>TPL</t>
+        </is>
+      </c>
+      <c r="Q238" t="n">
+        <v>0.7367</v>
+      </c>
+      <c r="R238" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="S238" t="n">
+        <v>0.6395</v>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="U238" t="n">
+        <v>0.6264</v>
+      </c>
+      <c r="V238" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="W238" t="n">
+        <v>0.6061</v>
+      </c>
+      <c r="X238" t="inlineStr">
+        <is>
+          <t>KEYS</t>
+        </is>
+      </c>
+      <c r="Y238" t="n">
+        <v>0.5577</v>
+      </c>
+      <c r="Z238" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AA238" t="n">
+        <v>0.5513</v>
+      </c>
+      <c r="AB238" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="AC238" t="n">
+        <v>0.5228</v>
+      </c>
+      <c r="AD238" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="AE238" t="n">
+        <v>0.5193</v>
+      </c>
+      <c r="AF238" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+      <c r="AG238" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="AH238" t="inlineStr">
+        <is>
+          <t>TRGP</t>
+        </is>
+      </c>
+      <c r="AI238" t="n">
+        <v>0.4675</v>
+      </c>
+      <c r="AJ238" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="AK238" t="n">
+        <v>0.4505</v>
+      </c>
+      <c r="AL238" t="inlineStr">
+        <is>
+          <t>EQIX</t>
+        </is>
+      </c>
+      <c r="AM238" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="AN238" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="AO238" t="n">
+        <v>0.4334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update data 2026/04/23 週四
</commit_message>
<xml_diff>
--- a/rebalance_holdings_final.xlsx
+++ b/rebalance_holdings_final.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I238"/>
+  <dimension ref="A1:I239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11612,6 +11612,53 @@
       <c r="I238" t="inlineStr">
         <is>
           <t>22.03%</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>28.57%</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>24.41%</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>23.79%</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>23.22%</t>
         </is>
       </c>
     </row>
@@ -11626,7 +11673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO238"/>
+  <dimension ref="A1:AO239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51413,6 +51460,173 @@
       </c>
       <c r="AO238" t="n">
         <v>0.4334</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>0.9094</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>0.8945</v>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>0.8319</v>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="I239" t="n">
+        <v>0.7871</v>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="K239" t="n">
+        <v>0.7862</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="M239" t="n">
+        <v>0.7524999999999999</v>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="O239" t="n">
+        <v>0.7149</v>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="Q239" t="n">
+        <v>0.6909</v>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="S239" t="n">
+        <v>0.6571</v>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>KEYS</t>
+        </is>
+      </c>
+      <c r="U239" t="n">
+        <v>0.6483</v>
+      </c>
+      <c r="V239" t="inlineStr">
+        <is>
+          <t>TPL</t>
+        </is>
+      </c>
+      <c r="W239" t="n">
+        <v>0.5878</v>
+      </c>
+      <c r="X239" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="Y239" t="n">
+        <v>0.5832000000000001</v>
+      </c>
+      <c r="Z239" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="AA239" t="n">
+        <v>0.5787</v>
+      </c>
+      <c r="AB239" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="AC239" t="n">
+        <v>0.5541</v>
+      </c>
+      <c r="AD239" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="AE239" t="n">
+        <v>0.5264</v>
+      </c>
+      <c r="AF239" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+      <c r="AG239" t="n">
+        <v>0.4996</v>
+      </c>
+      <c r="AH239" t="inlineStr">
+        <is>
+          <t>EQIX</t>
+        </is>
+      </c>
+      <c r="AI239" t="n">
+        <v>0.4549</v>
+      </c>
+      <c r="AJ239" t="inlineStr">
+        <is>
+          <t>TRGP</t>
+        </is>
+      </c>
+      <c r="AK239" t="n">
+        <v>0.4257</v>
+      </c>
+      <c r="AL239" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="AM239" t="n">
+        <v>0.4112</v>
+      </c>
+      <c r="AN239" t="inlineStr">
+        <is>
+          <t>COP</t>
+        </is>
+      </c>
+      <c r="AO239" t="n">
+        <v>0.4022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update data 2026/04/30 週四
</commit_message>
<xml_diff>
--- a/rebalance_holdings_final.xlsx
+++ b/rebalance_holdings_final.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I239"/>
+  <dimension ref="A1:I240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11659,6 +11659,53 @@
       <c r="I239" t="inlineStr">
         <is>
           <t>23.22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>29.13%</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>24.65%</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>24.23%</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>21.98%</t>
         </is>
       </c>
     </row>
@@ -11673,7 +11720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO239"/>
+  <dimension ref="A1:AO240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51627,6 +51674,173 @@
       </c>
       <c r="AO239" t="n">
         <v>0.4022</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>GLW</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>0.9397</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>0.8642</v>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>LYB</t>
+        </is>
+      </c>
+      <c r="G240" t="n">
+        <v>0.8192</v>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>0.8046</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>0.7635999999999999</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="M240" t="n">
+        <v>0.7423999999999999</v>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="O240" t="n">
+        <v>0.7337</v>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>KEYS</t>
+        </is>
+      </c>
+      <c r="Q240" t="n">
+        <v>0.7257</v>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S240" t="n">
+        <v>0.7067</v>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="U240" t="n">
+        <v>0.6318</v>
+      </c>
+      <c r="V240" t="inlineStr">
+        <is>
+          <t>GEV</t>
+        </is>
+      </c>
+      <c r="W240" t="n">
+        <v>0.6254</v>
+      </c>
+      <c r="X240" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="Y240" t="n">
+        <v>0.6181</v>
+      </c>
+      <c r="Z240" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="AA240" t="n">
+        <v>0.5966</v>
+      </c>
+      <c r="AB240" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="AC240" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="AD240" t="inlineStr">
+        <is>
+          <t>VLO</t>
+        </is>
+      </c>
+      <c r="AE240" t="n">
+        <v>0.4987</v>
+      </c>
+      <c r="AF240" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="AG240" t="n">
+        <v>0.4746</v>
+      </c>
+      <c r="AH240" t="inlineStr">
+        <is>
+          <t>EQIX</t>
+        </is>
+      </c>
+      <c r="AI240" t="n">
+        <v>0.4718</v>
+      </c>
+      <c r="AJ240" t="inlineStr">
+        <is>
+          <t>PWR</t>
+        </is>
+      </c>
+      <c r="AK240" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="AL240" t="inlineStr">
+        <is>
+          <t>MPC</t>
+        </is>
+      </c>
+      <c r="AM240" t="n">
+        <v>0.4257</v>
+      </c>
+      <c r="AN240" t="inlineStr">
+        <is>
+          <t>TPL</t>
+        </is>
+      </c>
+      <c r="AO240" t="n">
+        <v>0.4166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>